<commit_message>
feature: added alter the message
</commit_message>
<xml_diff>
--- a/whatsapp.xlsx
+++ b/whatsapp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saeedbinsalman/Documents/repos/whatsapp-sender/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42BCDFD1-0EAE-3648-B4CD-D3CAC538B193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553188B4-A9ED-564C-98C2-F7C734EA2102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15820" xr2:uid="{DD9C563E-B14B-3A4F-8C05-92AE6B257E49}"/>
   </bookViews>
@@ -53,10 +53,10 @@
     <t>سعيد عمر</t>
   </si>
   <si>
-    <t>صباح الخير</t>
+    <t>0559368234</t>
   </si>
   <si>
-    <t>0559368234</t>
+    <t>hi</t>
   </si>
 </sst>
 </file>
@@ -153,13 +153,13 @@
         <xdr:from>
           <xdr:col>3</xdr:col>
           <xdr:colOff>749300</xdr:colOff>
-          <xdr:row>4</xdr:row>
+          <xdr:row>3</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>5</xdr:col>
           <xdr:colOff>622300</xdr:colOff>
-          <xdr:row>5</xdr:row>
+          <xdr:row>4</xdr:row>
           <xdr:rowOff>177800</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
@@ -536,11 +536,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B59B99EB-E23F-7943-A6E7-90E250340F84}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17.83203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="38.33203125" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -559,10 +559,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -594,11 +594,6 @@
       <c r="A8" s="2"/>
       <c r="B8" s="3"/>
       <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -616,13 +611,13 @@
                   <from>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>749300</xdr:colOff>
-                    <xdr:row>4</xdr:row>
+                    <xdr:row>3</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>5</xdr:col>
                     <xdr:colOff>622300</xdr:colOff>
-                    <xdr:row>5</xdr:row>
+                    <xdr:row>4</xdr:row>
                     <xdr:rowOff>177800</xdr:rowOff>
                   </to>
                 </anchor>

</xml_diff>

<commit_message>
ft: ability to reconnect to whatsapp
</commit_message>
<xml_diff>
--- a/whatsapp.xlsx
+++ b/whatsapp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saeedbinsalman/Documents/repos/whatsapp-sender/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553188B4-A9ED-564C-98C2-F7C734EA2102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8411AC98-06B3-A340-A218-DDFBDA4A13E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15820" xr2:uid="{DD9C563E-B14B-3A4F-8C05-92AE6B257E49}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>الرساله</t>
   </si>
@@ -57,6 +57,12 @@
   </si>
   <si>
     <t>hi</t>
+  </si>
+  <si>
+    <t>+12064897489</t>
+  </si>
+  <si>
+    <t>hihi</t>
   </si>
 </sst>
 </file>
@@ -567,8 +573,12 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="2"/>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>

</xml_diff>